<commit_message>
Added Calls page for observability
</commit_message>
<xml_diff>
--- a/ReceptionistData.xlsx
+++ b/ReceptionistData.xlsx
@@ -1066,7 +1066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1115,6 +1115,11 @@
           <t>end_time</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>session_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1254,6 +1259,58 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>252954de</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-08T12:31:32</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Logan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2033594344</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2af03d6a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding stylest and service
</commit_message>
<xml_diff>
--- a/ReceptionistData.xlsx
+++ b/ReceptionistData.xlsx
@@ -8,10 +8,10 @@
   <sheets>
     <sheet name="Hours" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Location" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Services" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Associates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Schedule" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Appointments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Appointments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Services" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Associates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Schedule" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -665,76 +665,304 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>duration_minutes</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>customer_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>customer_phone</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stylist</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>end_time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>session_id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>7128bd8e</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-25T13:10:38</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Test Caller</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+15551234</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Joey</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Cut</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C2" t="n">
-        <v>35</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>90</v>
-      </c>
-      <c r="C3" t="n">
-        <v>95</v>
+          <t>1c2cf840</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-29T10:38:20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Logan Deliberto</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2033594344</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Joey</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>120</v>
-      </c>
-      <c r="C4" t="n">
-        <v>120</v>
+          <t>8f5836f8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-29T11:12:22</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Logan Deliberto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2033594344</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mandy</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shave</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>30</v>
-      </c>
-      <c r="C5" t="n">
-        <v>25</v>
+          <t>252954de</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-08T12:31:32</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Logan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2033594344</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2af03d6a</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>08c377ea</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-08T12:55:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Logan D'Iberto</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2037890351</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Trim</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ebfcc39c</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -748,117 +976,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Service 1</t>
+          <t>duration_minutes</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Service 2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Service 3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Service 4</t>
+          <t>price</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Delores</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>Cut</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
+      <c r="B2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Joey</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Cut</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Shave</t>
-        </is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C3" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mandy</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Cut</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Shave</t>
-        </is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>120</v>
+      </c>
+      <c r="C4" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sam</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Cut</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
           <t>Shave</t>
         </is>
+      </c>
+      <c r="B5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Trim</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -872,43 +1072,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Service 1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Service 2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Service 3</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Saturday</t>
+          <t>Service 4</t>
         </is>
       </c>
     </row>
@@ -918,29 +1108,14 @@
           <t>Delores</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10AM to 4PM</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10AM to 4PM</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10AM to 4PM</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>10AM to 4PM</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>10AM to 4PM</t>
+          <t>Perm</t>
         </is>
       </c>
     </row>
@@ -950,34 +1125,14 @@
           <t>Joey</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>12PM to 6PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>12PM to 6PM</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>12PM to 6PM</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>12PM to 7PM</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>12PM to 6PM</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>12PM to 5PM</t>
+          <t>Shave</t>
         </is>
       </c>
     </row>
@@ -987,34 +1142,19 @@
           <t>Mandy</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10AM to 3PM</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10AM to 3PM</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10AM to 3PM</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10AM to 7PM</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>10AM to 3PM</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>10AM to 3PM</t>
+          <t>Shave</t>
         </is>
       </c>
     </row>
@@ -1024,34 +1164,46 @@
           <t>Sam</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1PM to 6PM</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1PM to 6PM</t>
+          <t>Perm</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1PM to 6PM</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1PM to 7PM</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>1PM to 6PM</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>1PM to 5PM</t>
+          <t>Shave</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Shave</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Trim</t>
         </is>
       </c>
     </row>
@@ -1066,251 +1218,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>customer_name</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>customer_phone</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>stylist</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>start_time</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>end_time</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>session_id</t>
+          <t>Saturday</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7128bd8e</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-25T13:10:38</t>
+          <t>Delores</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Test Caller</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>+15551234</t>
+          <t>10AM to 4PM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Joey</t>
+          <t>10AM to 4PM</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>10AM to 4PM</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>10AM to 4PM</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>13:30</t>
+          <t>10AM to 4PM</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1c2cf840</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-29T10:38:20</t>
+          <t>Joey</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Logan Deliberto</t>
+          <t>12PM to 6PM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2033594344</t>
+          <t>12PM to 6PM</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Joey</t>
+          <t>12PM to 6PM</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>12PM to 7PM</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>12PM to 6PM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>13:30</t>
+          <t>12PM to 5PM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8f5836f8</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-29T11:12:22</t>
+          <t>Mandy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Logan Deliberto</t>
+          <t>10AM to 3PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2033594344</t>
+          <t>10AM to 3PM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mandy</t>
+          <t>10AM to 3PM</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>10AM to 7PM</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>10AM to 3PM</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>12:00</t>
+          <t>10AM to 3PM</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>252954de</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-07-08T12:31:32</t>
+          <t>Sam</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Logan</t>
+          <t>1PM to 6PM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2033594344</t>
+          <t>1PM to 6PM</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>1PM to 6PM</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>1PM to 7PM</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>1PM to 6PM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2af03d6a</t>
+          <t>1PM to 5PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10AM to 5PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10AM to 5PM</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>10AM to 5PM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10AM to 5PM</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10AM to 5PM</t>
         </is>
       </c>
     </row>

</xml_diff>